<commit_message>
Add Data Quality Dashboard, data-file Copilot, PD Investment, resizable tables
New Data_Quality.aspx (21 rules, multi-select filters, issues pop-up, notes,
daily tracking) with Home tile and menu entry. Copilot reads every data file
and answers on any column/filter. Scorecard tables gain Capital Investment
and PD Investment. Tab icon on all pages; tables fit, columns and boxes resize.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/pipeline-fixture.xlsx
+++ b/tests/fixtures/pipeline-fixture.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI125"/>
+  <dimension ref="A1:AK125"/>
   <sheetData>
     <row r="1">
       <c r="D1" t="str">
@@ -524,6 +524,12 @@
       <c r="AI5" t="str">
         <v>Total Investment (OPEX+CAPEX)</v>
       </c>
+      <c r="AJ5" t="str">
+        <v>Capital Investment</v>
+      </c>
+      <c r="AK5" t="str">
+        <v>Product Development Investment</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -625,6 +631,12 @@
       <c r="AI6">
         <v>1565308</v>
       </c>
+      <c r="AJ6">
+        <v>547858</v>
+      </c>
+      <c r="AK6">
+        <v>782654</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -726,6 +738,12 @@
       <c r="AI7">
         <v>2131014</v>
       </c>
+      <c r="AJ7">
+        <v>745855</v>
+      </c>
+      <c r="AK7">
+        <v>1065507</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -824,6 +842,12 @@
       <c r="AI8">
         <v>2345662</v>
       </c>
+      <c r="AJ8">
+        <v>820982</v>
+      </c>
+      <c r="AK8">
+        <v>1172831</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -916,6 +940,12 @@
       <c r="AI9">
         <v>2234736</v>
       </c>
+      <c r="AJ9">
+        <v>782158</v>
+      </c>
+      <c r="AK9">
+        <v>1117368</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -1017,6 +1047,12 @@
       <c r="AI10">
         <v>667463</v>
       </c>
+      <c r="AJ10">
+        <v>233612</v>
+      </c>
+      <c r="AK10">
+        <v>333732</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -1115,6 +1151,12 @@
       <c r="AI11">
         <v>2180650</v>
       </c>
+      <c r="AJ11">
+        <v>763228</v>
+      </c>
+      <c r="AK11">
+        <v>1090325</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -1216,6 +1258,12 @@
       <c r="AI12">
         <v>751952</v>
       </c>
+      <c r="AJ12">
+        <v>263183</v>
+      </c>
+      <c r="AK12">
+        <v>375976</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -1317,6 +1365,12 @@
       <c r="AI13">
         <v>510991</v>
       </c>
+      <c r="AJ13">
+        <v>178847</v>
+      </c>
+      <c r="AK13">
+        <v>255496</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -1418,6 +1472,12 @@
       <c r="AI14">
         <v>131467</v>
       </c>
+      <c r="AJ14">
+        <v>46013</v>
+      </c>
+      <c r="AK14">
+        <v>65734</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -1519,6 +1579,12 @@
       <c r="AI15">
         <v>754273</v>
       </c>
+      <c r="AJ15">
+        <v>263996</v>
+      </c>
+      <c r="AK15">
+        <v>377137</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -1617,6 +1683,12 @@
       <c r="AI16">
         <v>2154543</v>
       </c>
+      <c r="AJ16">
+        <v>754090</v>
+      </c>
+      <c r="AK16">
+        <v>1077272</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -1718,6 +1790,12 @@
       <c r="AI17">
         <v>964323</v>
       </c>
+      <c r="AJ17">
+        <v>337513</v>
+      </c>
+      <c r="AK17">
+        <v>482162</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -1816,6 +1894,12 @@
       <c r="AI18">
         <v>1599679</v>
       </c>
+      <c r="AJ18">
+        <v>559888</v>
+      </c>
+      <c r="AK18">
+        <v>799840</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -1908,6 +1992,12 @@
       <c r="AI19">
         <v>2178843</v>
       </c>
+      <c r="AJ19">
+        <v>762595</v>
+      </c>
+      <c r="AK19">
+        <v>1089422</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -2006,6 +2096,12 @@
       <c r="AI20">
         <v>606029</v>
       </c>
+      <c r="AJ20">
+        <v>212110</v>
+      </c>
+      <c r="AK20">
+        <v>303015</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -2107,6 +2203,12 @@
       <c r="AI21">
         <v>398505</v>
       </c>
+      <c r="AJ21">
+        <v>139477</v>
+      </c>
+      <c r="AK21">
+        <v>199253</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -2208,6 +2310,12 @@
       <c r="AI22">
         <v>1168322</v>
       </c>
+      <c r="AJ22">
+        <v>408913</v>
+      </c>
+      <c r="AK22">
+        <v>584161</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -2309,6 +2417,12 @@
       <c r="AI23">
         <v>792018</v>
       </c>
+      <c r="AJ23">
+        <v>277206</v>
+      </c>
+      <c r="AK23">
+        <v>396009</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -2401,6 +2515,12 @@
       <c r="AI24">
         <v>1038845</v>
       </c>
+      <c r="AJ24">
+        <v>363596</v>
+      </c>
+      <c r="AK24">
+        <v>519423</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -2493,6 +2613,12 @@
       <c r="AI25">
         <v>2471100</v>
       </c>
+      <c r="AJ25">
+        <v>864885</v>
+      </c>
+      <c r="AK25">
+        <v>1235550</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -2594,6 +2720,12 @@
       <c r="AI26">
         <v>1422220</v>
       </c>
+      <c r="AJ26">
+        <v>497777</v>
+      </c>
+      <c r="AK26">
+        <v>711110</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -2686,6 +2818,12 @@
       <c r="AI27">
         <v>2162628</v>
       </c>
+      <c r="AJ27">
+        <v>756920</v>
+      </c>
+      <c r="AK27">
+        <v>1081314</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -2787,6 +2925,12 @@
       <c r="AI28">
         <v>1929620</v>
       </c>
+      <c r="AJ28">
+        <v>675367</v>
+      </c>
+      <c r="AK28">
+        <v>964810</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -2888,6 +3032,12 @@
       <c r="AI29">
         <v>883627</v>
       </c>
+      <c r="AJ29">
+        <v>309269</v>
+      </c>
+      <c r="AK29">
+        <v>441814</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -2986,6 +3136,12 @@
       <c r="AI30">
         <v>333704</v>
       </c>
+      <c r="AJ30">
+        <v>116796</v>
+      </c>
+      <c r="AK30">
+        <v>166852</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -3078,6 +3234,12 @@
       <c r="AI31">
         <v>2260832</v>
       </c>
+      <c r="AJ31">
+        <v>791291</v>
+      </c>
+      <c r="AK31">
+        <v>1130416</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -3173,6 +3335,12 @@
       <c r="AI32">
         <v>280442</v>
       </c>
+      <c r="AJ32">
+        <v>98155</v>
+      </c>
+      <c r="AK32">
+        <v>140221</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -3265,6 +3433,12 @@
       <c r="AI33">
         <v>1194876</v>
       </c>
+      <c r="AJ33">
+        <v>418207</v>
+      </c>
+      <c r="AK33">
+        <v>597438</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -3357,6 +3531,12 @@
       <c r="AI34">
         <v>2399819</v>
       </c>
+      <c r="AJ34">
+        <v>839937</v>
+      </c>
+      <c r="AK34">
+        <v>1199910</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -3449,6 +3629,12 @@
       <c r="AI35">
         <v>547341</v>
       </c>
+      <c r="AJ35">
+        <v>191569</v>
+      </c>
+      <c r="AK35">
+        <v>273671</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -3550,6 +3736,12 @@
       <c r="AI36">
         <v>1807356</v>
       </c>
+      <c r="AJ36">
+        <v>632575</v>
+      </c>
+      <c r="AK36">
+        <v>903678</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -3651,6 +3843,12 @@
       <c r="AI37">
         <v>253415</v>
       </c>
+      <c r="AJ37">
+        <v>88695</v>
+      </c>
+      <c r="AK37">
+        <v>126708</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -3752,6 +3950,12 @@
       <c r="AI38">
         <v>1970872</v>
       </c>
+      <c r="AJ38">
+        <v>689805</v>
+      </c>
+      <c r="AK38">
+        <v>985436</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -3853,6 +4057,12 @@
       <c r="AI39">
         <v>886673</v>
       </c>
+      <c r="AJ39">
+        <v>310336</v>
+      </c>
+      <c r="AK39">
+        <v>443337</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -3951,6 +4161,12 @@
       <c r="AI40">
         <v>2177724</v>
       </c>
+      <c r="AJ40">
+        <v>762203</v>
+      </c>
+      <c r="AK40">
+        <v>1088862</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -4052,6 +4268,12 @@
       <c r="AI41">
         <v>95738</v>
       </c>
+      <c r="AJ41">
+        <v>33508</v>
+      </c>
+      <c r="AK41">
+        <v>47869</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -4144,6 +4366,12 @@
       <c r="AI42">
         <v>899354</v>
       </c>
+      <c r="AJ42">
+        <v>314774</v>
+      </c>
+      <c r="AK42">
+        <v>449677</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -4236,6 +4464,12 @@
       <c r="AI43">
         <v>455257</v>
       </c>
+      <c r="AJ43">
+        <v>159340</v>
+      </c>
+      <c r="AK43">
+        <v>227629</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -4337,6 +4571,12 @@
       <c r="AI44">
         <v>2061612</v>
       </c>
+      <c r="AJ44">
+        <v>721564</v>
+      </c>
+      <c r="AK44">
+        <v>1030806</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -4438,6 +4678,12 @@
       <c r="AI45">
         <v>1741370</v>
       </c>
+      <c r="AJ45">
+        <v>609480</v>
+      </c>
+      <c r="AK45">
+        <v>870685</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -4539,6 +4785,12 @@
       <c r="AI46">
         <v>471703</v>
       </c>
+      <c r="AJ46">
+        <v>165096</v>
+      </c>
+      <c r="AK46">
+        <v>235852</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -4640,6 +4892,12 @@
       <c r="AI47">
         <v>1511689</v>
       </c>
+      <c r="AJ47">
+        <v>529091</v>
+      </c>
+      <c r="AK47">
+        <v>755845</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -4741,6 +4999,12 @@
       <c r="AI48">
         <v>1916620</v>
       </c>
+      <c r="AJ48">
+        <v>670817</v>
+      </c>
+      <c r="AK48">
+        <v>958310</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -4830,6 +5094,12 @@
       <c r="AI49">
         <v>467131</v>
       </c>
+      <c r="AJ49">
+        <v>163496</v>
+      </c>
+      <c r="AK49">
+        <v>233566</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -4928,6 +5198,12 @@
       <c r="AI50">
         <v>2478794</v>
       </c>
+      <c r="AJ50">
+        <v>867578</v>
+      </c>
+      <c r="AK50">
+        <v>1239397</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -5026,6 +5302,12 @@
       <c r="AI51">
         <v>1576304</v>
       </c>
+      <c r="AJ51">
+        <v>551706</v>
+      </c>
+      <c r="AK51">
+        <v>788152</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -5118,6 +5400,12 @@
       <c r="AI52">
         <v>1229742</v>
       </c>
+      <c r="AJ52">
+        <v>430410</v>
+      </c>
+      <c r="AK52">
+        <v>614871</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -5219,6 +5507,12 @@
       <c r="AI53">
         <v>63008</v>
       </c>
+      <c r="AJ53">
+        <v>22053</v>
+      </c>
+      <c r="AK53">
+        <v>31504</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -5311,6 +5605,12 @@
       <c r="AI54">
         <v>2297536</v>
       </c>
+      <c r="AJ54">
+        <v>804138</v>
+      </c>
+      <c r="AK54">
+        <v>1148768</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -5400,6 +5700,12 @@
       <c r="AI55">
         <v>720830</v>
       </c>
+      <c r="AJ55">
+        <v>252290</v>
+      </c>
+      <c r="AK55">
+        <v>360415</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -5492,6 +5798,12 @@
       <c r="AI56">
         <v>280102</v>
       </c>
+      <c r="AJ56">
+        <v>98036</v>
+      </c>
+      <c r="AK56">
+        <v>140051</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -5581,6 +5893,12 @@
       <c r="AI57">
         <v>1556120</v>
       </c>
+      <c r="AJ57">
+        <v>544642</v>
+      </c>
+      <c r="AK57">
+        <v>778060</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -5679,6 +5997,12 @@
       <c r="AI58">
         <v>1835519</v>
       </c>
+      <c r="AJ58">
+        <v>642432</v>
+      </c>
+      <c r="AK58">
+        <v>917760</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -5768,6 +6092,12 @@
       <c r="AI59">
         <v>43503</v>
       </c>
+      <c r="AJ59">
+        <v>15226</v>
+      </c>
+      <c r="AK59">
+        <v>21752</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -5866,6 +6196,12 @@
       <c r="AI60">
         <v>303367</v>
       </c>
+      <c r="AJ60">
+        <v>106178</v>
+      </c>
+      <c r="AK60">
+        <v>151684</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -5967,6 +6303,12 @@
       <c r="AI61">
         <v>2373816</v>
       </c>
+      <c r="AJ61">
+        <v>830836</v>
+      </c>
+      <c r="AK61">
+        <v>1186908</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -6059,6 +6401,12 @@
       <c r="AI62">
         <v>177323</v>
       </c>
+      <c r="AJ62">
+        <v>62063</v>
+      </c>
+      <c r="AK62">
+        <v>88662</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -6160,6 +6508,12 @@
       <c r="AI63">
         <v>1524765</v>
       </c>
+      <c r="AJ63">
+        <v>533668</v>
+      </c>
+      <c r="AK63">
+        <v>762383</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -6258,6 +6612,12 @@
       <c r="AI64">
         <v>755352</v>
       </c>
+      <c r="AJ64">
+        <v>264373</v>
+      </c>
+      <c r="AK64">
+        <v>377676</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -6350,6 +6710,12 @@
       <c r="AI65">
         <v>1332163</v>
       </c>
+      <c r="AJ65">
+        <v>466257</v>
+      </c>
+      <c r="AK65">
+        <v>666082</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -6448,6 +6814,12 @@
       <c r="AI66">
         <v>745535</v>
       </c>
+      <c r="AJ66">
+        <v>260937</v>
+      </c>
+      <c r="AK66">
+        <v>372768</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -6546,6 +6918,12 @@
       <c r="AI67">
         <v>2234166</v>
       </c>
+      <c r="AJ67">
+        <v>781958</v>
+      </c>
+      <c r="AK67">
+        <v>1117083</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -6647,6 +7025,12 @@
       <c r="AI68">
         <v>720430</v>
       </c>
+      <c r="AJ68">
+        <v>252150</v>
+      </c>
+      <c r="AK68">
+        <v>360215</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -6736,6 +7120,12 @@
       <c r="AI69">
         <v>1028707</v>
       </c>
+      <c r="AJ69">
+        <v>360047</v>
+      </c>
+      <c r="AK69">
+        <v>514354</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -6837,6 +7227,12 @@
       <c r="AI70">
         <v>1258787</v>
       </c>
+      <c r="AJ70">
+        <v>440575</v>
+      </c>
+      <c r="AK70">
+        <v>629394</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -6938,6 +7334,12 @@
       <c r="AI71">
         <v>1064450</v>
       </c>
+      <c r="AJ71">
+        <v>372558</v>
+      </c>
+      <c r="AK71">
+        <v>532225</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -7039,6 +7441,12 @@
       <c r="AI72">
         <v>1807487</v>
       </c>
+      <c r="AJ72">
+        <v>632620</v>
+      </c>
+      <c r="AK72">
+        <v>903744</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -7140,6 +7548,12 @@
       <c r="AI73">
         <v>1303452</v>
       </c>
+      <c r="AJ73">
+        <v>456208</v>
+      </c>
+      <c r="AK73">
+        <v>651726</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -7241,6 +7655,12 @@
       <c r="AI74">
         <v>965954</v>
       </c>
+      <c r="AJ74">
+        <v>338084</v>
+      </c>
+      <c r="AK74">
+        <v>482977</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -7339,6 +7759,12 @@
       <c r="AI75">
         <v>2002201</v>
       </c>
+      <c r="AJ75">
+        <v>700770</v>
+      </c>
+      <c r="AK75">
+        <v>1001101</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -7431,6 +7857,12 @@
       <c r="AI76">
         <v>1926864</v>
       </c>
+      <c r="AJ76">
+        <v>674402</v>
+      </c>
+      <c r="AK76">
+        <v>963432</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -7523,6 +7955,12 @@
       <c r="AI77">
         <v>1354483</v>
       </c>
+      <c r="AJ77">
+        <v>474069</v>
+      </c>
+      <c r="AK77">
+        <v>677242</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -7618,6 +8056,12 @@
       <c r="AI78">
         <v>910784</v>
       </c>
+      <c r="AJ78">
+        <v>318774</v>
+      </c>
+      <c r="AK78">
+        <v>455392</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -7707,6 +8151,12 @@
       <c r="AI79">
         <v>2319258</v>
       </c>
+      <c r="AJ79">
+        <v>811740</v>
+      </c>
+      <c r="AK79">
+        <v>1159629</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -7796,6 +8246,12 @@
       <c r="AI80">
         <v>900789</v>
       </c>
+      <c r="AJ80">
+        <v>315276</v>
+      </c>
+      <c r="AK80">
+        <v>450395</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81">
@@ -7894,6 +8350,12 @@
       <c r="AI81">
         <v>411846</v>
       </c>
+      <c r="AJ81">
+        <v>144146</v>
+      </c>
+      <c r="AK81">
+        <v>205923</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82">
@@ -7995,6 +8457,12 @@
       <c r="AI82">
         <v>886482</v>
       </c>
+      <c r="AJ82">
+        <v>310269</v>
+      </c>
+      <c r="AK82">
+        <v>443241</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83">
@@ -8096,6 +8564,12 @@
       <c r="AI83">
         <v>1904548</v>
       </c>
+      <c r="AJ83">
+        <v>666592</v>
+      </c>
+      <c r="AK83">
+        <v>952274</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84">
@@ -8194,6 +8668,12 @@
       <c r="AI84">
         <v>1435007</v>
       </c>
+      <c r="AJ84">
+        <v>502252</v>
+      </c>
+      <c r="AK84">
+        <v>717504</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85">
@@ -8295,6 +8775,12 @@
       <c r="AI85">
         <v>693381</v>
       </c>
+      <c r="AJ85">
+        <v>242683</v>
+      </c>
+      <c r="AK85">
+        <v>346691</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -8384,6 +8870,12 @@
       <c r="AI86">
         <v>1188309</v>
       </c>
+      <c r="AJ86">
+        <v>415908</v>
+      </c>
+      <c r="AK86">
+        <v>594155</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -8476,6 +8968,12 @@
       <c r="AI87">
         <v>225302</v>
       </c>
+      <c r="AJ87">
+        <v>78856</v>
+      </c>
+      <c r="AK87">
+        <v>112651</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88">
@@ -8577,6 +9075,12 @@
       <c r="AI88">
         <v>266328</v>
       </c>
+      <c r="AJ88">
+        <v>93215</v>
+      </c>
+      <c r="AK88">
+        <v>133164</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89">
@@ -8678,6 +9182,12 @@
       <c r="AI89">
         <v>1662356</v>
       </c>
+      <c r="AJ89">
+        <v>581825</v>
+      </c>
+      <c r="AK89">
+        <v>831178</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90">
@@ -8779,6 +9289,12 @@
       <c r="AI90">
         <v>274374</v>
       </c>
+      <c r="AJ90">
+        <v>96031</v>
+      </c>
+      <c r="AK90">
+        <v>137187</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91">
@@ -8877,6 +9393,12 @@
       <c r="AI91">
         <v>2382015</v>
       </c>
+      <c r="AJ91">
+        <v>833705</v>
+      </c>
+      <c r="AK91">
+        <v>1191008</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92">
@@ -8978,6 +9500,12 @@
       <c r="AI92">
         <v>440532</v>
       </c>
+      <c r="AJ92">
+        <v>154186</v>
+      </c>
+      <c r="AK92">
+        <v>220266</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93">
@@ -9079,6 +9607,12 @@
       <c r="AI93">
         <v>886029</v>
       </c>
+      <c r="AJ93">
+        <v>310110</v>
+      </c>
+      <c r="AK93">
+        <v>443015</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94">
@@ -9165,6 +9699,12 @@
       <c r="AI94">
         <v>1236950</v>
       </c>
+      <c r="AJ94">
+        <v>432933</v>
+      </c>
+      <c r="AK94">
+        <v>618475</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95">
@@ -9266,6 +9806,12 @@
       <c r="AI95">
         <v>1634044</v>
       </c>
+      <c r="AJ95">
+        <v>571915</v>
+      </c>
+      <c r="AK95">
+        <v>817022</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96">
@@ -9364,6 +9910,12 @@
       <c r="AI96">
         <v>961048</v>
       </c>
+      <c r="AJ96">
+        <v>336367</v>
+      </c>
+      <c r="AK96">
+        <v>480524</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97">
@@ -9465,6 +10017,12 @@
       <c r="AI97">
         <v>1352373</v>
       </c>
+      <c r="AJ97">
+        <v>473331</v>
+      </c>
+      <c r="AK97">
+        <v>676187</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98">
@@ -9563,6 +10121,12 @@
       <c r="AI98">
         <v>2445424</v>
       </c>
+      <c r="AJ98">
+        <v>855898</v>
+      </c>
+      <c r="AK98">
+        <v>1222712</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99">
@@ -9655,6 +10219,12 @@
       <c r="AI99">
         <v>1224425</v>
       </c>
+      <c r="AJ99">
+        <v>428549</v>
+      </c>
+      <c r="AK99">
+        <v>612213</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -9756,6 +10326,12 @@
       <c r="AI100">
         <v>920738</v>
       </c>
+      <c r="AJ100">
+        <v>322258</v>
+      </c>
+      <c r="AK100">
+        <v>460369</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101">
@@ -9857,6 +10433,12 @@
       <c r="AI101">
         <v>1935096</v>
       </c>
+      <c r="AJ101">
+        <v>677284</v>
+      </c>
+      <c r="AK101">
+        <v>967548</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102">
@@ -9955,6 +10537,12 @@
       <c r="AI102">
         <v>1098496</v>
       </c>
+      <c r="AJ102">
+        <v>384474</v>
+      </c>
+      <c r="AK102">
+        <v>549248</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103">
@@ -10056,6 +10644,12 @@
       <c r="AI103">
         <v>116309</v>
       </c>
+      <c r="AJ103">
+        <v>40708</v>
+      </c>
+      <c r="AK103">
+        <v>58155</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104">
@@ -10148,6 +10742,12 @@
       <c r="AI104">
         <v>403176</v>
       </c>
+      <c r="AJ104">
+        <v>141112</v>
+      </c>
+      <c r="AK104">
+        <v>201588</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105">
@@ -10249,6 +10849,12 @@
       <c r="AI105">
         <v>194750</v>
       </c>
+      <c r="AJ105">
+        <v>68163</v>
+      </c>
+      <c r="AK105">
+        <v>97375</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106">
@@ -10350,6 +10956,12 @@
       <c r="AI106">
         <v>683767</v>
       </c>
+      <c r="AJ106">
+        <v>239318</v>
+      </c>
+      <c r="AK106">
+        <v>341884</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107">
@@ -10448,6 +11060,12 @@
       <c r="AI107">
         <v>2236986</v>
       </c>
+      <c r="AJ107">
+        <v>782945</v>
+      </c>
+      <c r="AK107">
+        <v>1118493</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108">
@@ -10549,6 +11167,12 @@
       <c r="AI108">
         <v>473225</v>
       </c>
+      <c r="AJ108">
+        <v>165629</v>
+      </c>
+      <c r="AK108">
+        <v>236613</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109">
@@ -10650,6 +11274,12 @@
       <c r="AI109">
         <v>1928024</v>
       </c>
+      <c r="AJ109">
+        <v>674808</v>
+      </c>
+      <c r="AK109">
+        <v>964012</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110">
@@ -10748,6 +11378,12 @@
       <c r="AI110">
         <v>940337</v>
       </c>
+      <c r="AJ110">
+        <v>329118</v>
+      </c>
+      <c r="AK110">
+        <v>470169</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111">
@@ -10849,6 +11485,12 @@
       <c r="AI111">
         <v>1893413</v>
       </c>
+      <c r="AJ111">
+        <v>662695</v>
+      </c>
+      <c r="AK111">
+        <v>946707</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112">
@@ -10941,6 +11583,12 @@
       <c r="AI112">
         <v>771310</v>
       </c>
+      <c r="AJ112">
+        <v>269959</v>
+      </c>
+      <c r="AK112">
+        <v>385655</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113">
@@ -11042,6 +11690,12 @@
       <c r="AI113">
         <v>1714576</v>
       </c>
+      <c r="AJ113">
+        <v>600102</v>
+      </c>
+      <c r="AK113">
+        <v>857288</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114">
@@ -11134,6 +11788,12 @@
       <c r="AI114">
         <v>1994779</v>
       </c>
+      <c r="AJ114">
+        <v>698173</v>
+      </c>
+      <c r="AK114">
+        <v>997390</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115">
@@ -11235,6 +11895,12 @@
       <c r="AI115">
         <v>717527</v>
       </c>
+      <c r="AJ115">
+        <v>251134</v>
+      </c>
+      <c r="AK115">
+        <v>358764</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116">
@@ -11336,6 +12002,12 @@
       <c r="AI116">
         <v>2130164</v>
       </c>
+      <c r="AJ116">
+        <v>745557</v>
+      </c>
+      <c r="AK116">
+        <v>1065082</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117">
@@ -11437,6 +12109,12 @@
       <c r="AI117">
         <v>1924908</v>
       </c>
+      <c r="AJ117">
+        <v>673718</v>
+      </c>
+      <c r="AK117">
+        <v>962454</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118">
@@ -11538,6 +12216,12 @@
       <c r="AI118">
         <v>1398345</v>
       </c>
+      <c r="AJ118">
+        <v>489421</v>
+      </c>
+      <c r="AK118">
+        <v>699173</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119">
@@ -11630,6 +12314,12 @@
       <c r="AI119">
         <v>654431</v>
       </c>
+      <c r="AJ119">
+        <v>229051</v>
+      </c>
+      <c r="AK119">
+        <v>327216</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120">
@@ -11731,6 +12421,12 @@
       <c r="AI120">
         <v>60530</v>
       </c>
+      <c r="AJ120">
+        <v>21186</v>
+      </c>
+      <c r="AK120">
+        <v>30265</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121">
@@ -11832,6 +12528,12 @@
       <c r="AI121">
         <v>2104602</v>
       </c>
+      <c r="AJ121">
+        <v>736611</v>
+      </c>
+      <c r="AK121">
+        <v>1052301</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122">
@@ -11921,6 +12623,12 @@
       <c r="AI122">
         <v>2029231</v>
       </c>
+      <c r="AJ122">
+        <v>710231</v>
+      </c>
+      <c r="AK122">
+        <v>1014616</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123">
@@ -12013,6 +12721,12 @@
       <c r="AI123">
         <v>394536</v>
       </c>
+      <c r="AJ123">
+        <v>138088</v>
+      </c>
+      <c r="AK123">
+        <v>197268</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124">
@@ -12102,6 +12816,12 @@
       <c r="AI124">
         <v>226742</v>
       </c>
+      <c r="AJ124">
+        <v>79360</v>
+      </c>
+      <c r="AK124">
+        <v>113371</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125">
@@ -12203,10 +12923,16 @@
       <c r="AI125">
         <v>2084180</v>
       </c>
+      <c r="AJ125">
+        <v>729463</v>
+      </c>
+      <c r="AK125">
+        <v>1042090</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AI125"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AK125"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>